<commit_message>
import as pdf features has been added
</commit_message>
<xml_diff>
--- a/chat_log.xlsx
+++ b/chat_log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,832 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-07 16:52:11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hi how are you , how can you help me</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hola, estoy muy bien, gracias por preguntar. 😊  
+Como asistente especializado en el contexto proporcionado (que contiene registros detallados de reuniones de lobby del Instituto de Salud Pública de Chile), puedo ayudarte específicamente con información extraída de esas audiencias. Por ejemplo, puedo:  
+- Detallar **fechas, horarios y plataformas** de reuniones específicas (como las de Guido Álvarez el 23/01/2026 o Sergio Muñoz el 05/05/2026).  
+- Explicar los **temas discutidos** en cada reunión (ej.: "Diseño, implementación y evaluación de políticas", "Celebración o modificación de contratos", o "Elaboración de actos administrativos").  
+- Proporcionar datos sobre **participantes** (gestores de intereses, empresas representadas, como WAYS Asesorías Ltda., Tres HTP Professional Services SPA, o Consultorías Públicas Ltda.).  
+- Compartir **identificadores de reunión** (AO005AW2049774, AO005AW2104542, etc.) y **enlaces de origen** para verificarlos directamente en leylobby.gob.cl.  
+- Resumir **propósitos clave** mencionados en las solicitudes (ej.: presentación de soluciones de ciberseguridad como Kymatio, plataformas de gestión documental como FEBOS, o consultas sobre trámites pendientes en SIAC).  
+Para darte una respuesta precisa y útil, ¿podrías especificar qué aspecto de estas reuniones te interesa? Por ejemplo:  
+- ¿Quieres saber sobre reuniones relacionadas con **ciberseguridad** (como la de WAYS Asesorías Ltda. del 23/01/2026)?  
+- ¿Necesitas detalles sobre **trámites de contratación o modificaciones de contratos** (tema recurrente en múltiples entradas)?  
+- ¿Te gustaría conocer información sobre **gestión de productos farmacéuticos** (reuniones de Guisela Isabel Zurich Reszczynski o Sergio Muñoz)?  
+- ¿Hay 15 reuniones documentadas en el contexto—estoy aquí para ayudarte a navegar esa información con exactitud. ¡Adelante con tu pregunta! 📋✨</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-08 14:29:44</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>What specific concern did Ana María Araya Figueroa express regarding the Chillán Hospital and pembrolizumab treatment for patients with triple-negative breast cancer?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Based on a thorough review of the provided context containing all meeting records from January to May 2026, there is **no mention** of:
+- Ana María Araya Figueroa
+- Chillán Hospital
+- Pembrolizumab
+- Triple-negative breast cancer
+The context includes detailed records of 20 meetings discussing various regulatory matters such as:
+- Implementation of new therapies for colorectal cancer hepatic metastases
+- Authorization of clinical trials for pediatric leukemia
+- Advanced therapy projects (R-MATIS)
+- Pharmaceutical product registrations and biosimilars
+- Device regulation and hazardous product labeling
+- Clinical study approval processes
+- Specific product discussions (Cyramza, Pluvicto, Opdivo, etc.)
+None of these meetings contain any reference to the specific elements in your query. The context focuses exclusively on pharmaceutical regulation, clinical trial authorizations, device regulation, and related administrative processes within Chile's healthcare system, but does not include any discussion about breast cancer treatments, pembrolizumab, or concerns raised by individuals named Ana María Araya Figueroa regarding Chillán Hospital.
+Therefore, I cannot provide information about Ana María Araya Figueroa's specific concern regarding Chillán Hospital and pembrolizumab treatment for triple-negative breast cancer, as this topic is not addressed in the provided context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-08 14:44:10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>What specific concern did Ana María Araya Figueroa express regarding the Chillán Hospital</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ana María Araya Figueroa expressed the following specific concern regarding the Hospital de Chillán:  
+**"El Hospital de Chillán está dejando fuera del tratamiento a pacientes que, por criterio de resultado de biopsia, sí debieran recibir Pembrolizumab. Sin embargo, les están indicando Tamoxifeno."**  
+This translates to:  
+*The Chillán Hospital is excluding patients from treatment who, based on biopsy results, should receive Pembrolizumab. However, they are being indicated Tamoxifen instead.*  
+This concern was raised during the videoconferencia meeting on **May 19, 2026 at 10:00 AM**, where Ana María Araya Figueroa (representing herself as a Gestor de intereses) discussed issues related to cancer treatment access, specifically highlighting the Chillán Hospital's deviation from appropriate Pembrolizumab prescribing practices for eligible triple-negative breast cancer patients.  
+**Key details from the context:**  
+- The concern was part of her broader explanation about challenges in cancer care access, including delays in pembrolizumab distribution and resource limitations in other hospitals (La Serena, Sótero del Río, Van Buren).  
+- She emphasized that while pembrolizumab has been available since the October 2025 RE DAC update, its timely delivery remains inconsistent, and the Chillán Hospital's practice of substituting Tamoxifen for Pembrolizumab in biopsy-eligible patients represents a critical clinical discrepancy.  
+- This issue was presented to Alejandro Berkovits (Jefe Agencia Nacional del Cáncer, SSP) during the meeting focused on *"Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos."*  
+No other mentions of the Chillán Hospital appear in the provided context, making this the sole and specific concern attributed to Ana María Araya Figueroa regarding this institution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-08 14:59:07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>what happens on meet in On May 19, 2026 at 10:00 AM, Alejandro Berkovits</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está lo que ocurrió en la reunión del **19 de mayo de 2026 a las 10:00 AM** con Alejandro Berkovits:
+- **Participante principal**: ANA MARIA ARAYA FIGUEROA (representando a sí misma como gestora de intereses) asistió a la videoconferencia mediante el enlace Zoom: https://minsal-cl.zoom.us/j/85649906536 (contraseña: 323352).
+- **Duración**: La reunión duró exactamente 1 hora (1 horas, 0 minutos).
+- **Tema central**: Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos.
+- **Propósito y detalles de la discusión**:
+  - Ana María Araya Figueroa expuso sus preocupaciones específicas sobre el tratamiento de pacientes con **cáncer de mama triple negativo**.
+  - Señaló que, aunque el medicamento **pembrolizumab** está disponible desde la resolución que actualizó la RE DAC en octubre de 2025, **su entrega no siempre es oportuna**, lo que retrasa el tratamiento de las pacientes.
+  - Mencionó que la distribución del medicamento se ha **centralizado**, lo que ha reducido los tiempos de espera en comparación con períodos anteriores.
+  - Expresó preocupación por la **gestión y falta de recursos** en los hospitales de **La Serena, Sótero del Río y Van Buren**, lo que afecta la atención oncológica.
+  - Destacó un problema crítico en el **Hospital de Chillán**: está **excluyendo del tratamiento con pembrolizumab** a pacientes que, según el resultado de su biopsia, **sí deberían recibirlo**, indicándoles en su lugar **tamoxifeno** (un tratamiento inadecuado para este subtipo de cáncer).
+  - A nivel personal, informó que planeaba presentarse ante la **Comisión de Mujeres y Equidad de Género** y la **Comisión de Salud** (coordinada por dos parlamentarios), y que le habría gustado compartir estos detalles directamente con el Dr. Berkovits.
+  - Consultó sobre tres temas adicionales:
+    1. La disponibilidad de **asesoramiento genético** para pacientes.
+    2. La posible **actualización de las canastas GES** específicamente para el cáncer de mama.
+    3. Si el **recorte presupuestario en salud** afectaría el financiamiento de drogas o la atención de los pacientes.
+  - En relación con su última consulta, se le informó oficialmente que **ningún recorte presupuestario afectará directamente la atención de las personas**, pero se le sugirió **reiterar todas sus consultas (incluyendo las anteriores) mediante el mecanismo de Transparencia**, donde recibiría una respuesta más detallada en un plazo de algunos días.
+- **Identificador de la reunión**: AO001AW2179080.
+- **Fuente oficial**: https://www.leylobby.gob.cl/instituciones/AO001/audiencias/2026/903081/911908.
+En resumen, la reunión se centró en los desafíos de acceso oportuno al pembrolizumab para cáncer de mama triple negativo, problemas de gestión hospitalaria específicos, y consultas sobre políticas públicas relacionadas con el tratamiento oncológico, con orientación oficial para usar canales de transparencia para seguimiento detallado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-08 15:06:33</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">who is Alejandro Berkovits
+</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, Alejandro Berkovits es el **Jefe de la Agencia Nacional del Cáncer, SSP** (Subsecretaría de Salud Pública o equivalente dentro del Ministerio de Salud de Chile). 
+Esta información se menciona de manera consistente en todos los registros de reuniones incluidos en el contexto, donde se le identifica siempre como:
+- "Alejandro Berkovits, the Jefe Agencia Nacional del Cáncer, SSP"
+- Asistiendo a videoconferencias oficiales relacionadas con temas de políticas oncológicas, diseño e implementación de programas de salud, y otros asuntos vinculados al control y prevención del cáncer en Chile.
+Su rol implica participar en reuniones con gestores de intereses, representantes de organizaciones y fundaciones para discutir asuntos relacionados con el cáncer, incluyendo acceso a tratamientos, políticas públicas, gestión hospitalaria y avances en investigación oncológica, como se evidencia en las múltiples audiencias detalladas en el contexto (por ejemplo, las reuniones del 19 de mayo de 2026, 29 de mayo de 2026, 28 de mayo de 2026, entre otras). 
+No se proporciona información adicional sobre su formación académica, trayectoria previa o detalles personales más allá de su cargo oficial en el contexto dado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-08 15:36:49</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">what happens on meet in On May 19, 2026 at 10:00 AM, Alejandro Berkovits
+</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está lo que ocurrió en la reunión del **19 de mayo de 2026 a las 10:00 AM** donde Alejandro Berkovits (Jefe Agencia Nacional del Cáncer, SSP) participó como asistente:
+### 📋 **Detalles clave de la reunión:**
+- **Identificador de la reunión:** AO001AW2179080  
+- **Plataforma:** Videoconferencia mediante Zoom (Enlace: https://minsal-cl.zoom.us/j/85649906536, Contraseña: 323352)  
+- **Duración:** 1 hora, 0 minutos  
+- **Tema principal discutido:** *Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos*  
+- **Participante destacado:** ANA MARIA ARAYA FIGUEROA (Gestor de intereses, trabajando para *nan*, representando a **Ana María Araya**)  
+- **Enlace de origen:** https://www.leylobby.gob.cl/instituciones/AO001/audiencias/2026/903081/911908  
+---
+### 💬 **¿Qué se discutió en la reunión?**  
+Ana María Araya Figueroa expuso las siguientes preocupaciones y solicitudes al Ministerio de Salud (representado por Alejandro Berkovits):  
+#### 1️⃣ **Problemas con el acceso al pembrolizumab para cáncer de mama triple negativo:**  
+- Aunque el medicamento **pembrolizumab** está disponible desde la resolución que actualizó la **RE DAC en octubre de 2025**, su entrega **no siempre llega a tiempo**, lo que retrasa el tratamiento de las pacientes.  
+- Señaló que, aunque la distribución se ha **centralizado** y ahora **demora menos que antes**, persisten retrasos críticos.  
+#### 2️⃣ **Preocupaciones por gestión y recursos hospitalarios:**  
+- Expresó inquietud por la **falta de recursos y gestión deficiente** en los hospitales de:  
+  - **La Serena**  
+  - **Sótero del Río**  
+  - **Van Buren**  
+- Destacó un caso específico: el **Hospital de Chillán** está **excluyendo indebidamente** a pacientes que, según el resultado de su biopsia, **deberían recibir pembrolizumab**, indicándoles en su lugar **tamoxifeno** (un tratamiento menos adecuado para este subtipo de cáncer).  
+#### 3️⃣ **Planos personales y de incidencia política:**  
+- Mencionó que planea presentarse ante:  
+  - La **Comisión de Mujeres y Equidad de Género**  
+  - La **Comisión de Salud** (coordinada por dos parlamentarios)  
+- Indicó que le habría gustado informar personalmente al Dr. Berkovits sobre estos temas antes de sus comparecencias.  
+#### 4️⃣ **Consultas adicionales planteadas:**  
+Ana María también preguntó sobre:  
+- **Asesoramiento genético** para pacientes oncológicos.  
+- **Posible actualización de las canastas GES** específicamente para el cáncer de mama.  
+- **Impacto del recorte presupuestario en salud** sobre:  
+  - El financiamiento de drogas oncológicas.  
+  - La atención integral de los pacientes.  
+#### 5️⃣ **Respuesta del Ministerio (según se le comunicó a Ana María):**  
+- Se le aclaró que, **oficialmente**, el Ministerio de Salud ha señalado que **ningún recorte presupuestario afectará directamente la atención de las personas**.  
+- Sin embargo, se le **sugirió reiterar todas sus consultas** (incluyendo las mencionadas anteriormente) a través del mecanismo de **Transparencia**, ya que este canal permite obtener respuestas **más detalladas y documentadas** en un plazo de **unos días**.  
+---
+### �  
+---
+### 📌 **Conclusión de la reunión:**  
+La audiencia se centró en **brechas críticas en el acceso oportuno a tratamientos oncológicos específicos** (pembrolizumab para cáncer de mama triple negativo), **deficiencias en la ejecución hospitalaria** (caso del Hospital de Chillán) y **preocupaciones sistémicas** relacionadas con recursos, políticas públicas (GES) y financiamiento. Ana María buscó tanto información inmediata como canales formales para abordar estas questões a nivel institucional, con el Ministerio orientándola hacia la vía de Transparencia para seguimiento técnico detallado.  
+Esta reunión refleja los esfuerzos continuos por parte de representantes de la sociedad civil y pacientes para monitorear y mejorar la implementación de políticas oncológicas en Chile, especialmente en el contexto de la **Ley Nacional del Cáncer** y las garantías GES.  
+¿Desea que profundice en algún aspecto específico de esta reunión o en otras audiencias relacionadas con el cáncer de mama triple negativo o el pembrolizumab? 😊</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-08 15:43:01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>who are you</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Soy **AI Bot**, un asistente especializado diseñado para proporcionar respuestas precisas, detalladas y basadas exclusivamente en el contexto y el historial de chat proporcionados. Mi función es analizar la información recuperada para ofrecer respuestas exhaustivas, interactivas y alineadas con las instrucciones específicas del sistema, sin utilizar conocimientos externos ni pre-entrenados. 
+Si tienes más preguntas sobre las reuniones, documentos o temas mencionados en el contexto (como la audiencia del 19 de mayo de 2026 con Alejandro Berkovits), estaré encantado de ayudarte con un análisis profundo y estructurado. 😊</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-08 15:46:25</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Could you please provide the details regarding the cancer-related meetings? I would like to know what is being discussed.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí tienes un análisis detallado de las reuniones relacionadas con el cáncer, incluyendo qué se discutió en cada una. He excluido la reunión del 24 de abril de 2026 a las 08:45 AM (sobre internet satelital en zonas remotas) ya que no está directamente relacionada con temas oncológicos, enfocándome exclusivamente en aquellas que abordan políticas, tratamientos, acceso a mediciones o iniciativas específicas contra el cáncer.
+---
+### 🎯 **Temas centrales recurrentes en las reuniones oncológicas**
+A lo largo de las audiencias registradas, se observan varios ejes de discusión persistentes:
+- **Acceso y distribución de medicamentos oncológicos innovadores** (pembrolizumab, sacituzumab, nivolumab/ipilimumab, luspatercept, dostarlimab, teclistamab, daratumumab, toripalimab).
+- **Desafíos en la implementación hospitalaria** (retrasos en entrega de fármacos, falta de recursos, decisiones clínicas inapropiadas como el uso de tamoxifeno en lugar de pembrolizumab en el Hospital de Chillán).
+- **Integración de ensayos clínicos y innovación tecnológica** (proyectos piloto, dispositivos de detección temprana como "Celbrea", plataformas de diagnóstico como RED VIRPATH y GESFIX).
+- **Actualización de marcos regulatorios y de cobertura** (modificaciones a las canastas GES, resolución DAC, Ley Nacional del Cáncer).
+- **Colaboración público-privada** (interés de laboratorios y centros de investigación en establecer acuerdos de riesgo compartido, redes de prestadores y alianzas con establecimientos asistenciales).
+- **Impacto económico y presupuestario** (proyecciones de costos, ahorros potenciales, preocupaciones por recortes y su efecto en financiamiento de drogas y atención integral).
+- **Participación de la sociedad civil y defensa de pacientes** (intervenciones de fundaciones, agrupaciones oncológicas y representantes de pacientes en comisiones y mesas de trabajo).
+---
+### 📅 **Resumen cronológico de las reuniones oncológicas clave**
+#### 🔹 **10 de marzo de 2026, 15:00**  
+- **Participante:** Carolina Ibáñez Cáceres (representando a sí misma).  
+- **Funcionario presente:** Sung Kim (Jefe de Agencia Nacional de Prevención y Control del Cáncer ANACAN).  
+- **Temas discutidos:**  
+  - Necesidades actuales en cáncer ginecológicos en el sistema de salud chileno.  
+  - Registro de tumores ginecológicos en UC y HSR, con especial preocupación por el cáncer de endometrio.  
+  - Priorización técnica desde ANACAN para incluir el cáncer de endometrio en las Garantías Explícitas en Salud (GES).  
+  - Contacto con referentes técnicos para avanzar en la propuesta.  
+#### 🔹 **25 de marzo de 2026, 03:30** (reunión presencial)  
+- **Funcionaria presente:** May Chomali Garib (Ministra de Salud).  
+- **Participantes:** Representantes de Fundación Cancer Vida, Observatorio del Cáncer, Corporación Valientes y Fundación Oncologica La Voz de los Pacientes Chile.  
+- **Temas discutidos:**  
+  - Listas de espera en cáncer.  
+  - Alternativas terapéuticas de primera línea en cáncer.  
+  - Registro nacional de cáncer.  
+  - Mesa de trabajo con la sociedad civil.  
+#### 🔹 **16 de abril de 2026, 10:00**  
+- **Participante:** Andrés Arellano (representando a PACIFIC GENOMICS SPA).  
+- **Funcionario presente:** Alejandro Berkovits (Jefe Agencia Nacional del Cáncer, SSP).  
+- **Temas discutidos:**  
+  - Iniciativa para implementar soluciones diagnósticas en el sistema de salud público (en fase avanzada de desarrollo, con definiciones técnicas y administrativas establecidas).  
+  - Revisión del estado de avance, identificación de acciones pendientes y coordinación de continuidad.  
+  - Modelo de implementación basado en coordinación centralizada para procesamiento y análisis, con articulación a nivel nacional.  
+  - Elementos del flujo operativo: evaluación técnica, procesamiento de muestras, entrega de resultados mediante plataformas seguras para profesionales de salud.  
+  - Estado contractual (en proceso de revisión para formalización conforme a normativa vigente).  
+  - **Acuerdos:** Definición de punto de contacto para coordinación, designación de contraparte técnica para supervisión, elaboración de cronograma de trabajo y entrega de antecedentes necesarios.  
+#### 🔹 **17 de abril de 2026, 08:00**  
+- **Participantes:** Jenny Henríquez, Luis Santiago y Patricio Araya (representando a PEGASI DE CHILE SpA).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Iniciativa de salud digital para mejorar la gestión clínica y continuidad de atención en pacientes oncológicos.  
+  - Enfoque en integración de información clínica, optimización de procesos asistenciales y uso de herramientas tecnológicas para apoyo en toma de decisiones.  
+  - Modelo de trabajo basado en plataformas digitales para automatización de flujos, estandarización de procesos clínicos y seguimiento longitudinal de pacientes.  
+  - Experiencias piloto y validaciones en distintos contextos para fortalecer detección oportuna y mejorar eficiencia en la atención.  
+  - Uso de metodologías basadas en datos para facilitar coordinación entre equipos clínicos y mejorar oportunidad de prestaciones de salud.  
+  - Aspectos generales de implementación: aplicación progresiva, articulación con establecimientos de salud y resguardo de estándares adecuados en gestión de información.  
+#### 🔹 **24 de abril de 2026, 08:00**  
+- **Participantes:** Jorge Rodrigo Martínez Moya, Orieta Matus y Álvaro Ibarra Valencia (representando a Instituto de Anatomía Patológica Dra. Virginia Martínez Corta SpA).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Presentación de iniciativas para fortalecer diagnóstico oportuno del cáncer y reducir listas de espera GES.  
+  - **RED VIRPATH:** Plataforma que utiliza tecnología e inteligencia artificial aplicada a anatomía patológica para acelerar diagnósticos oncológicos.  
+  - **GESFIX:** Plataforma destinada a optimizar gestión de capacidades y procesos del sistema de salud para disminuir listas de espera, con impacto escalable a nivel nacional.  
+#### 🔹 **29 de abril de 2026, 12:00**  
+- **Participantes:** Mariella Parodi, Juan Sebastian Robledo Arango y Carolina Beltran (representando a GlaxoSmithKline Chile Farmacéutica Ltda).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Presentación de evidencia científica relacionada con el uso de dostarlimab en cáncer de endometrio.  
+  - Antecedentes clínicos y terapéuticos asociados a su utilización en el manejo oncológico de esta patología.  
+#### 🔹 **29 de abril de 2026, 16:30**  
+- **Participante:** Jorge Fernández (representando a Asociación Chilena de Agrupaciones Oncológicas - ACHAGO).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Presentación de ACHAGO como organización representativa de agrupaciones de pacientes oncológicos a nivel nacional.  
+  - Participación en la implementación de la Ley Nacional del Cáncer y en la Comisión Nacional del Cáncer.  
+  - Diálogo sobre desafíos asociados a la alerta sanitaria oncológica vigente.  
+  - Posibles instancias de colaboración con el Ministerio de Salud en materia de participación ciudadana y fortalecimiento de la respuesta oncológica a nivel territorial.  
+#### 🔹 **8 de mayo de 2026, 09:20**  
+- **Participantes:** Marco Ojier (Profemlab spa), Andrea Ojier, Alicia Barbosa y Jorge Salazar (algunos marcados como "nan" para entidad empleadora).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Presentación de “Celbrea”: dispositivo portátil no invasivo orientado a fortalecer la detección temprana del cáncer de mama mediante nanosensores termográficos.  
+  - Potencial uso como herramienta complementaria de priorización en Atención Primaria de Salud para optimizar derivaciones y disminuir listas de espera para mamografías.  
+  - Consultas respecto a funcionamiento, utilidad clínica y continuidad diagnóstica.  
+  - Interés en explorar oportunidades de colaboración público-privada en materia de prevención y detección oportuna del cáncer de mama.  
+#### 🔹 **14 de mayo de 2026, 08:00**  
+- **Participantes:** Natalia Celedón, Lorena Vega, Amanda Caetano Batista, Sandra Monteiro y Mauricio Cuadra (representando a Merck Sharp and Dohme).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Mauricio Cuadra presentó a Merck como laboratorio número uno en investigación en Chile (productos en vacunas, inmunoterapia - Keytruda como producto estrella, enfermedades cardio metabólicas y raras).  
+  - Reafirmación de compromiso con el Ministerio de Salud en el desafío contra el cáncer cérvico uterino mediante la vacuna VPH.  
+  - Cierre del convenio ARC para cáncer de mama triple negativo (CMTN) con pembrolizumab.  
+  - Desarrollo de una presentación subcutánea de pembrolizumab, próxima a comercializarse.  
+  - Lorena Vega presentó proyecto piloto con municipalidad de La Pintana para entrega de vacuna contra el VPH, ampliando población beneficiaria inicial a personas mayores de 9 años.  
+#### 🔹 **15 de mayo de 2026, 08:30**  
+- **Participantes:** Loreto Vidal (Gador Ltda), Nancy Oses (Bristol-Myers Squibb de Chile) y Teresa Vanegas (Gador Ltda).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Presentación de Sacituzumab Govitecan Trodelvy para tratamiento de cáncer de mama triple negativo (CMTN):  
+    - Indicado para adultos con CMTN irresecable o metastásico que hayan recibido ≥2 tratamientos sistémicos previos (incluyendo al menos uno para enfermedad avanzada).  
+    - También indicado para cáncer de mama HR+/HER2- irresecable o metastásico después de terapia endocrina y ≥2 tratamientos sistémicos adicionales en estadio avanzado.  
+    - Autorizado por el ISP desde febrero de 2025 para ambas indicaciones.  
+  - Resultados del estudio ASCENT (fase III):  
+    - Supervivencia libre de progresión (SLP): 5.4 meses vs 1.7 meses (quimioterapia estándar).  
+    - Supervivencia global (SG): 12.1 meses vs 6.7 meses.  
+    - Seguridad: 51% presentó neutropenia severa, 21% diarrea; sin muertes durante el estudio.  
+  - Proyección de costos a 3 años para 231 pacientes elegibles.  
+  - Plan de Gador para piloto en dos hospitales públicos (Barros Luco y Hospital de La Serena) incorporando tratamiento para CMTN en etapa metastásica.  
+#### 🔹 **19 de mayo de 2026, 10:00**  
+- **Participante:** Ana María Araya Figueroa (representando a sí misma).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - **Problemas de acceso al pembrolizumab para CMTN:**  
+    - Aunque disponible desde resolución DAC actualizada en octubre de 2025, su entrega no siempre llega a tiempo, retrasando tratamiento.  
+    - Distribución centralizada ha reducido demoras, pero persisten retrasos críticos.  
+  - **Preocupaciones por gestión y recursos hospitalarios:**  
+    - Falta de recursos y gestión deficiente en hospitales de La Serena, Sótero del Río y Van Buren.  
+    - Caso específico: Hospital de Chillán excluyendo indebidamente a pacientes que, según biopsia, deberían recibir pembrolizumab (indicándoles tamoxifeno en su lugar).  
+  - **Planos personales e institucionales:**  
+    - Intención de presentarse ante Comisión de Mujeres y Equidad de Género y Comisión de Salud (coordinada por dos parlamentarios).  
+    - Deseo de haber informado personalmente al Dr. Berkovits antes de sus comparecencias.  
+  - **Consultas adicionales:**  
+    - Asesoramiento genético para pacientes oncológicos.  
+    - Posible actualización de las canastas GES específicamente para cáncer de mama.  
+    - Impacto del recorte presupuestario en salud sobre financiamiento de drogas oncológicas y atención integral de pacientes.  
+  - **Respuesta del Ministerio:**  
+    - Oficialmente, ningún recorte presupuestario afectará directamente la atención de las personas.  
+    - Se sugirió reiterar consultas mediante mecanismo de Transparencia para obtener respuestas más detalladas y documentadas en unos días.  
+#### 🔹 **19 de mayo de 2026, 15:00**  
+- **Participante:** Elizabeth Mendoza (representando a Fundación en acción).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Exploración de alternativas para abordar situación de pacientes mastectomizadas por cáncer de mama en lista de espera para reconstrucción mamaria.  
+  - Gestiones previas con diversos Servicios de Salud sin resultados favorables.  
+  - Fundación cuenta con especialistas mastólogos dispuestos a realizar cirugías, pero carece de infraestructura necesaria (requiere apoyo y colaboración del Ministerio).  
+  - Durante la reunión, se le explicó a la interlocutora que consultas adicionales deben solicitarse mediante mecanismos establecidos por la Ley de Transparencia (no en instancia de lobby).  
+#### 🔹 **20 de mayo de 2026, 10:00**  
+- **Participantes:** Boris Álvarez y José Miguel Erpel Norambuena (representando a Centro de Oncología de Precisión SpA - Celerity).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Celerity cuenta con tres centros oncológicos en Iquique, Santiago y Concepción.  
+  - Interés en desarrollar proyecto piloto para modelo de colaboración y evaluar potencial contribución en marco de alerta sanitaria oncológica.  
+  - Disposición para impulsar propuesta colaborativa más amplia con principales centros de estudios clínicos del país.  
+  - Capacidad para favorecer continuidad de atención (sistema público y privado); reclutamiento mediante convenios institucionales o derivaciones de comités oncológicos.  
+  - Pacientes comparten información clínica con centro como parte de proceso de evaluación e incorporación.  
+  - Disponen de herramienta de prescreening para identificación y selección de potenciales pacientes candidatos a estudios clínicos.  
+  - **Acuerdos:** Celerity enviará presentación al Depto. del Cáncer; Francisca informará a jefatura acerca de la propuesta.  
+#### 🔹 **22 de mayo de 2026, 08:30**  
+- **Participantes:** Juan Corona y Alejandra Cisneros (representando a Bristol Myers Squibb).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - **Neoplasia mielodisplásica:**  
+    - Terapia Luspatercept Reblozyl: ~80% de pacientes desarrollan anemia y requieren transfusiones.  
+    - 60.4% de pacientes tratados con Reblozyl alcanzarían independencia transfusional.  
+    - Ahorro potencial estimado de 16.2 millones anuales por paciente.  
+    - Interés en explorar acuerdo de riesgo compartido con Ministerio de Salud.  
+  - **Cáncer colorrectal metastásico:**  
+    - Uso de Nivolumab Opdivo + Ipilimumab Yervoy.  
+    - Segundo cáncer en incidencia y tercero en mortalidad en Chile (10.6% de muertes por cáncer).  
+    - ~5% de casos corresponden a subtipo MSI-H/dMMR.  
+    - ~80% de pacientes tratados con combinación estarían vivos al cuarto año.  
+    - Reducción estimada del 84% en progresión de enfermedad cuando tratamiento es utilizado en primera línea.  
+    - Existe contrato vigente con CENABAST que ya contempla recursos asociados a nivolumab (facilitando incorporación sin costos adicionales).  
+  - **Cáncer pulmonar no microcítico:**  
+    - Uso de Nivolumab Opdivo + Ipilimumab Yervoy en combinación con quimioterapia.  
+    - Entre 20-30% de pacientes corresponden a variantes escamosas/non-escamosas sin acceso a inmunoterapia por no cumplir biomarcador PDL1 requerido.  
+    - Uno de cada cinco pacientes tratados con combinación en primera línea estaría vivo al quinto año.  
+    - Costo anual evitable estimado de aproximadamente 645 millones (podría aumentar a 813.5 millones al incorporar ahorros asociados a licencias médicas).  
+    - Interés en que estas indicaciones sean incorporadas junto con otras ya incluidas en última resolución DAC (específicamente en neoadyuvancia en pulmón y mesotelioma).  
+  - **Acuerdos:**  
+    - Paula Herrera compartirá antecedentes con Dr. Berkovits, Carolina Gómez y Pablo Skármeta (referentes técnicos vinculados a DAC, cáncer pulmonar y hematooncología).  
+    - Bristol Myers Squibb enviará presentación expuesta y estudios de evaluación económica.  
+    - Reiterada disposición para establecer acuerdos de riesgo financiero compartido con Ministerio de Salud.  
+#### 🔹 **27 de mayo de 2026, 15:00**  
+- **Participantes:** Juan Corona y Alejandra Cisneros (representando a Bristol Myers Squibb).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Se esperó 10 minutos la conexión del gestor de intereses; tras inasistencia, se dio por finalizada la espera.  
+  - **Tema:** Celebración, modificación o terminación a cualquier título de contratos necesarios para funcionamiento de sujetos pasivos.  
+#### 🔹 **28 de mayo de 2026, 08:00**  
+- **Participantes:** Hugo Aedo y Verónica Kramm (representando a Johnson &amp; Johnson Chile S.A).  
+- **Funcionario presente:** Alejandro Berkovits.  
+- **Temas discutidos:**  
+  - Presentación de tres productos del portafolio oncológico:  
+    - **Amivantamab:** Para cáncer de pulmón no células pequeñas (CPNCP) con mutaciones de inserción en exón 20 del EGFR.  
+      - Anticuerpo biespecífico EGFR/MET, aprobado en primera línea con carboplatino y pemetrexed para pacientes con CPNCP avanzado y mutación EGFR en exón 20.  
+      - Población objetivo: 112 de CPNCP con mutación EGFR (estimado 90.135 pacientes/año en Chile).  
+      - Duplica control de enfermedad frente a quimioterapia estándar, reduciendo eventos de progresión rápida y uso intensivo de recursos asistenciales.  
+    - **Teclistamab:** Para mieloma múltiple en recaída/refractario.  
+      - Anticuerpo biespecífico BCMA/CD3, siendo el primer biespecífico que une directamente célula tumoral con linfocito T del paciente.  
+      - Indicado en pacientes triple-expuestos (inmunomodulador, inhibidor del proteasoma, antiCD38).  
+      - Triplica control de enfermedad frente a alternativas estándar (SLP de 1112 meses vs 35 meses con terapia estándar).  
+      - Población objetivo en Chile estimada en 260.390 pacientes.  
+    - **Daratumumab:** Para mieloma múltiple.  
+      - Anticuerpo monoclonal antiCD38 que induce muerte tumoral por mecanismos inmunomediados.  
+      - Registro sanitario para múltiples indicaciones (primera línea y recaída/refractario).  
+      - Ventajas: único biológico aprobado en primera línea con respuestas profundas, duraderas y sostenidas; mediana de SLP proyectada en primera línea de 17 años; beneficio demostrado en alto riesgo citogenético; resultados comprobados en sector público y privado; disponible en formulación subcutánea.  
+  - Consultas:  
+    - Estudios nacionales o internacionales de impacto económico (no cuentan con estudios nacionales, pero harán averiguaciones por internacionales).  
+    - Postulación de tratamientos al DAC (se explicó que no existe postulación, sino priorización por comité respecto a problemas de salud oncológicos; este es medio para acercar terapias innovadoras al Departamento del Cáncer).  
+    - Cualquier solicitud de información adicional debe ser solicitada mediante ley de transparencia.  
+  - **Acuerdo:** Enviarán estudios y presentación realizada.  
+#### 🔹 **28 de mayo de 2026, 09:30**  
+- **Participantes:** Carlos Rojas, Federico Bakal, Constanza Parker y Maritza Huerta (representando a Bradford Hill Spa).  
+- **Funcionario presente:** Alejandro Berkovits (aunque no pudo asistir por razones de agenda).  
+- **Temas discutidos:**  
+  - Capacidad instalada para atención integral de pacientes oncológicos (laboratorio clínico, servicios de imágenes, oncología médica y otras especialidades de apoyo).  
+  - Disponibilidad de 24 sillones para infusión de quimioterapia y farmacia; capacidad para atender pacientes fuera de horarios destinados a estudios clínicos.  
+  - Interés en incorporar otros centros de investigación (especialmente en regiones) a una eventual red de atención para ampliar cobertura territorial y facilitar acceso a prestaciones oncológicas.  
+  - Manifestaron interés en integrarse a red de prestadores privados que participe en marco de alerta sanitaria oncológica (han realizado gestiones sin resultados favorables hasta la fecha).  
+  - Expresaron importancia de incorporar estudios clínicos dentro de políticas públicas relacionadas con cáncer (necesidad de fortalecer colaboración entre establecimientos asistenciales y centros de investigación mediante convenios).  
+  - **Descontento:** La audiencia fue solicitada para reunirse con Dr. Alejandro Berkovits, pero por razones de agenda no fue posible su participación.  
+#### 🔹 **29 de mayo de 2026, 08:45**  
+- **Participantes:** Carolina Zúñiga (representando a Dr Reddy`s Laboratories Chile SpA), Estefanía Castillo Vargas, Christian Rosales, Alex Matus y Felipe Zamora Rangel.  
+- **Funcionario presente:** Paula Herrera T. (en representación del Dr. Alejandro Berkovits, junto a representantes de DRL Chile y compañía internacional).  
+- **Temas discutidos:**  
+  - DRL presentó antecedentes sobre toripalimab para tratamiento de carcinoma nasofaríngeo y cáncer de esófago escamoso.  
+    - **Carcinoma nasofaríngeo:**  
+      - Baja incidencia en Chile, habitualmente diagnosticada en etapas avanzadas.  
+      - Toripalimab = anticuerpo monoclonal anti PD1 de segunda generación.  
+      - Resultados del estudio fase III JUPITER02: beneficios en sobrevida libre de progresión y sobrevida global a largo plazo.  
+      - Aprobado por agencias regulatorias internacionales (FDA, MHRA, EMA); incorporado en guías NCCN como tratamiento de primera línea.  
+    - **Cáncer de esófago escamoso:**  
+      - Antecedentes epidemiológicos nacionales.  
+      - Proporción importante de pacientes no cumple criterios de expresión de PDL1 requeridos para acceder a otras inmunoterapias aprobadas.  
+      - Resultados del estudio fase III JUPITER06: mejoras en sobrevida global para pacientes tratados con toripalimab en combinación con quimioterapia.  
+      - Beneficios observados serían independientes de expresión de PDL1 (considerado en aprobaciones regulatorias de MHRA y EMA).  
+  - **Acuerdos:**  
+    - Paula Herrera compartirá antecedentes presentados con Dr. Alejandro Berkovits y con Carolina Gómez (referente de DAC).  
+    - DRL se comprometió a enviar presentación expuesta durante la reunión para revisión y análisis.  
+---
+### 💡 **Conclusión general**
+Las reuniones revelan un esfuerzo activo por parte de laboratorios, centros de investigación, organizaciones de pacientes y autoridades sanitarias para:
+- **Avanzar en el acceso a terapias innovadoras** (inmunoterapias, anticuerpos biespecíficos, nuevos regímenes de quimioterapia).  
+- **Abordar brechas en la ejecución** (como los retrasos en pembrolizumab y decisiones clínicas inapropiadas en Hospital de Chillán).  
+- **Fortalecer el sistema mediante tecnología y colaboración** (plataformas de diagnóstico, proyectos piloto, redes de atención integrada).  
+- **Alinear innovación con políticas públicas** (actualización de GES, resolución DAC, incorporación de ensayos clínicos en estrategia nacional).  
+- **Garantizar sostenibilidad económica** mediante evaluaciones de costo-efectividad y exploración de modelos de riesgo compartido.  
+La participación de figuras clave como Alejandro Berkovits (Agencia Nacional del Cáncer) y Sung Kim (ANACAN) subraya el enfoque institucional en traducir estas discusiones en acciones concretas para mejorar la equidad, calidad y oportunidad en la atención oncológica en Chile.  
+¿Te gustaría que profundice en algún tema específico mencionado (por ejemplo, los detalles sobre el pembrolizumab en CMTN, los proyectos de diagnóstico como RED VIRPATH/GESFIX, o los acuerdos de riesgo compartido propuestos por las farmacéuticas)? Estoy aquí para proporcionar un análisis más focalizado según tus intereses. 😊</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:23:21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>what happens on meet in On May 19, 2026 at 10:00 AM, Alejandro Berkovits</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está lo que ocurrió en la reunión del **19 de mayo de 2026 a las 10:00 AM** con Alejandro Berkovits:
+**Detalles clave de la reunión:**
+- **Identificador de la reunión:** AO001AW2179080
+- **Plataforma:** Videoconferencia vía Zoom (Enlace: https://minsal-cl.zoom.us/j/85649906536, Contraseña: 323352)
+- **Duración:** 1 hora, 0 minutos
+- **Tema principal discutido:** Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos.
+**Propósito y contenido de la reunión:**
+La reunión fue solicitada por **Ana María Araya Figueroa** (representando a sí misma como gestora de intereses) para abordar preocupaciones específicas relacionadas con el acceso al tratamiento para pacientes con cáncer de mama triple negativo. Los puntos clave discutidos fueron:
+1. **Problemas de entrega del medicamento pembrolizumab:**
+   - Aunque el pembrolizumab se entrega desde la resolución que actualizó la RE DAC en octubre de 2025, su distribución aún presenta retrasos que afectan el tratamiento oportuno de las pacientes.
+   - Se mencionó que la distribución se ha centralizado, lo que ha reducido los tiempos de espera en comparación con períodos anteriores, pero persisten demoras significativas.
+2. **Preocupaciones sobre gestión y recursos hospitalarios:**
+   - Expresó inquietud por la gestión y falta de recursos en los hospitales de La Serena, Sótero del Río y Van Buren.
+   - Destacó específicamente que el Hospital de Chillán está excluyendo del tratamiento con pembrolizumab a pacientes que, según los resultados de biopsia, sí deberían recibir este medicamento, indicándoles en su lugar tamoxifeno (un tratamiento diferente y menos adecuado para este subtipo de cáncer).
+3. **Planos de participación institucional:**
+   - Informó que tiene previsto presentarse ante la Comisión de Mujeres y Equidad de Género y la Comisión de Salud (coordinada por dos parlamentarios), mencionando que le habría gustado informar personalmente al Dr. Berkovits sobre estos asuntos.
+4. **Consultas adicionales planteadas:**
+   - Sobre temas de asesoramiento genético para pacientes oncológicas.
+   - Sobre la posible actualización de las canastas GES (Garantías Explícitas en Salud) específicamente para el cáncer de mama.
+   - Sobre el impacto potencial de los recortes presupuestarios en salud en el financiamiento de drogas oncológicas y la atención general de los pacientes.
+**Respuesta del Ministerio de Salud (representado en la reunión):**
+- Se le informó a Ana María que, según la información oficial proporcionada por el Ministerio, **ningún recorte presupuestario afectará directamente la atención de las personas**.
+- Sin embargo, se le sugirió que **reitere todas sus consultas (incluyendo las mencionadas anteriormente) a través del mecanismo de Transparencia**, ya que este canal permitirá obtener respuestas más detalladas y documentadas en un plazo de algunos días.
+**Participante registrada:**
+- **ANA MARIA ARAYA FIGUEROA** (Gestor de intereses, working for nan, representing Ana María Araya)
+Esta reunión se centró exclusivamente en barreras de acceso al tratamiento oncológico específico para cáncer de mama triple negativo, destacando problemas logísticos de distribución de medicamentos clave y inconsistencias en la aplicación de protocolos clínicos entre diferentes establecimientos de salud pública.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:24:42</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>woh is Alejandro Berkovits</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Basado exclusivamente en el contexto proporcionado, Alejandro Berkovits es identificado de manera consistente en todas las reuniones documentadas como:
+**Jefe Agencia Nacional del Cáncer, SSP**  
+(Jefe de la Agencia Nacional del Cáncer, Subsecretaría de Salud Pública)
+Esta designación aparece en cada entrada de reunión donde participa, desde abril hasta mayo de 2026, incluyendo:
+- La reunión del 19 de mayo de 2026 a las 10:00 AM (AO001AW2179080)
+- Todas las demás audiencias listadas en el contexto (abril 16, abril 17, abril 21, abril 24, abril 29, mayo 7, mayo 8, mayo 14, mayo 15, mayo 19, mayo 20, mayo 22, mayo 27, mayo 28, mayo 29)
+El contexto no proporciona información adicional sobre su identidad personal (como formación académica, historial laboral previo o detalles biográficos más allá de su cargo oficial durante el período documentado). Toda la información disponible se limita a su rol institucional como máximo responsable de la Agencia Nacional del Cáncer dentro de la estructura del Ministerio de Salud de Chile, específicamente adscrito a la Subsecretaría de Salud Pública (SSP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:26:37</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>how are all participants in these above meetings</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está un desglose detallado de **todos los participantes externos** (gestores de intereses) en cada reunión documentada donde Alejandro Berkovits participó, organizada cronológicamente con toda la información específica disponible:
+---
+### **Reuniones de Febrero 2026**
+1. **11 de febrero de 2026, 04:30 PM**  
+   - **Reunión con:** Tania Herrera (Jefa División de Planificación Sanitaria)  
+   - **Participantes externos:**  
+     - Manuel Espinoza (Gestor de intereses, working for nan, representing AstraZeneca S.A.)  
+     - Francisco Pinto (Gestor de intereses, working for Laboratorio Astrazeneca, representing AstraZeneca S.A.)  
+     - Álvaro Sepúlveda (Gestor de intereses, working for Laboratorio Astrazeneca, representing AstraZeneca S.A.)  
+     - Natalia Gandolfi (Gestor de intereses, working for nan, representing AstraZeneca S.A.)  
+     - Maria Gabriela Chirino (Gestor de intereses, working for nan, representing AstraZeneca S.A.)  
+2. **17 de febrero de 2026, 03:30 PM**  
+   - **Reunión con:** Sung Kim (Jefe de Agencia Nacional de Prevención y Control del Cáncer ANACAN)  
+   - **Participantes externos:**  
+     - Sonia Torrealba (Gestor de intereses, working for Novartis Chile S.A, representing Novartis Chile S.A.)  
+     - Melanie Paccot (Gestor de intereses, working for Novartis Chile S.A, representing Novartis Chile S.A.)  
+---
+### **Reuniones de Abril 2026**
+3. **16 de abril de 2026, 10:00 AM**  
+   - **Plataforma:** Vía teams  
+   - **Participantes externos:**  
+     - Andrés Arellano (Gestor de intereses, working for PACIFIC GENOMICS SPA, representing Andres Arellano)  
+4. **17 de abril de 2026, 08:00 AM**  
+   - **Plataforma:** Zoom  
+   - **Participantes externos:**  
+     - Jenny Henríquez (Gestor de intereses, working for nan, representing PEGASI DE CHILE SpA)  
+     - Luis Santiago (Gestor de intereses, working for nan, representing PEGASI DE CHILE SpA)  
+     - Patricio Araya (Gestor de intereses, working for nan, representing PEGASI DE CHILE SpA)  
+5. **21 de abril de 2026, 10:30 AM**  
+   - **Plataforma:** Presencial  
+   - **Participantes externos:**  
+     - Digna González (Gestor de intereses, working for nan, representing Corporacion Valientes)  
+6. **24 de abril de 2026, 08:00 AM**  
+   - **Plataforma:** Zoom  
+   - **Participantes externos:**  
+     - Jorge Rodrigo Martínez Moya (Gestor de intereses, working for nan, representing Jorge Martínez Moya)  
+     - Orieta Matus (Gestor de intereses, working for sk medical, representing Orieta Matus Catalán)  
+     - Álvaro Ibarra Valencia (Gestor de intereses, working for nan, representing Álvaro Ibarra Valencia)  
+7. **29 de abril de 2026, 12:00 PM**  
+   - **Plataforma:** Zoom  
+   - **Participantes externos:**  
+     - Mariella Parodi (Gestor de intereses, working for GlaxoSmithKline Chile Farmacéutica Ltda, representing GlaxoSmithKline Chile Farmacéutica Ltda)  
+     - Juan Sebastian Robledo Arango (Gestor de intereses, working for GlaxoSmithKline Chile Farmacéutica Ltda, representing GlaxoSmithKline Chile Farmacéutica Ltda)  
+     - Carolina Beltran (Gestor de intereses, working for GlaxoSmithKline Chile Farmacéutica Ltda, representing GlaxoSmithKline Chile Farmacéutica Ltda)  
+8. **29 de abril de 2026, 04:30 PM**  
+   - **Plataforma:** Zoom  
+   - **Participantes externos:**  
+     - Jorge Fernández (Gestor de intereses, working for nan, representing Asociación Chilena de Agrupaciones Oncológicas)  
+---
+### **Reuniones de Mayo 2026**
+9. **08 de mayo de 2026, 08:45 AM**  
+   - **Plataforma:** Zoom  
+   - **Participantes externos:**  
+     - Sonia Torrealba (Gestor de intereses, working for Novartis Chile S.A, representing NOVARTIS CHILE S.A.)  
+     - LORETO RAMOS RODRIGUEZ (Gestor de intereses, working for nan, representing NOVARTIS CHILE S.A.)  
+10. **14 de mayo de 2026, 08:00 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Natalia Celedón (Gestor de intereses, working for nan, representing Merck Sharp and Dohme)  
+      - Lorena Vega (Gestor de intereses, working for Pfizer Chile SA, representing Merck Sharp and Dohme)  
+      - AMANDA CAETANO BATISTA (Gestor de intereses, working for nan, representing Merck Sharp and Dohme)  
+      - SANDRA MONTEIRO (Gestor de intereses, working for nan, representing Merck Sharp and Dohme)  
+      - Mauricio Cuadra (Gestor de intereses, working for nan, representing Merck Sharp and Dohme)  
+11. **15 de mayo de 2026, 08:30 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Loreto Vidal (Gestor de intereses, working for GADOR LTDA, representing GADOR Ltda)  
+      - Nancy Oses (Gestor de intereses, working for Bristol-Myers Squibb de Chile, representing GADOR Ltda)  
+      - Teresa Vanegas (Gestor de intereses, working for GADOR LTDA, representing GADOR Ltda)  
+12. **19 de mayo de 2026, 10:00 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - ANA MARIA ARAYA FIGUEROA (Gestor de intereses, working for nan, representing Ana María Araya)  
+13. **19 de mayo de 2026, 03:00 PM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Elizabeth Mendoza (Gestor de intereses, working for nan, representing Fundación en acción)  
+14. **20 de mayo de 2026, 08:00 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Jorge Fernández (Gestor de intereses, working for nan, representing Fundación de Ayuda a Personas con Cáncer ViDa)  
+15. **22 de mayo de 2026, 08:30 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Juan Corona (Gestor de intereses, working for nan, representing Bristol Myers Squibb)  
+      - Alejandra Cisneros (Gestor de intereses, working for Bristol-Myers Squibb de Chile, representing Bristol Myers Squibb)  
+16. **27 de mayo de 2026, 03:00 PM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Juan Corona (Gestor de intereses, working for nan, representing Bristol Myers Squibb)  
+      - Alejandra Cisneros (Gestor de intereses, working for Bristol-Myers Squibb de Chile, representing Bristol Myers Squibb)  
+17. **28 de mayo de 2026, 08:00 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Hugo Aedo (Gestor de intereses, working for Johnson &amp; Johnson, representing Johnson Johnson Chile S.A)  
+      - Verónica Kramm (Gestor de intereses, working for nan, representing Johnson Johnson Chile S.A)  
+18. **28 de mayo de 2026, 09:30 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Carlos Rojas (Gestor de intereses, working for nan, representing Bradford Hill Spa)  
+      - Federico Bakal (Gestor de intereses, working for nan, representing Bradford Hill Spa)  
+      - Constanza Parker (Gestor de intereses, working for nan, representing Bradford Hill Spa)  
+      - Maritza Huerta (Gestor de intereses, working for nan, representing Bradford Hill Spa)  
+19. **29 de mayo de 2026, 08:45 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Carolina Zúñiga (Gestor de intereses, working for Dr Reddy`s Laboratories Chile SpA, representing Carolina Zuñiga)  
+      - Estefanía Castillo Vargas (nan, working for nan, representing nan)  
+      - Christian Rosales (nan, working for nan, representing nan)  
+      - Alex Matus (nan, working for nan, representing nan)  
+      - Felipe Zamora Rangel (nan, working for nan, representing nan)  
+20. **29 de mayo de 2026, 09:00 AM**  
+    - **Plataforma:** Zoom  
+    - **Participantes externos:**  
+      - Boris Álvarez (Gestor de intereses, working for nan, representing Tecnigen SA)  
+---
+### **Observaciones clave sobre los participantes:**
+- **Repetición de participantes:** Algunas personas asistieron a múltiples reuniones, lo que indica intereses persistentes o seguimiento de temas específicos:  
+  - **Sonia Torrealba** (Novartis): Reuniones del 17/02 y 08/05  
+  - **Jorge Fernández** (Asociación Chilena de Agrupaciones Oncológicas / Fundación ViDa): Reuniones del 29/04 y 20/05  
+  - **Juan Corona y Alejandra Cisneros** (Bristol Myers Squibb): Reuniones del 22/05 y 27/05  
+- **Representaciones cruzadas:** En algunos casos, los participantes trabajaban para una empresa pero representaban a otra entidad (ej.: Nancy Oses trabajaba para Bristol-Myers Squibb pero representaba a GADOR Ltda el 15/05).  
+- **Diversidad de representantes:** Incluyeron:  
+  - Laboratorios farmacéuticos (Novartis, AstraZeneca, GlaxoSmithKline, Merck, Johnson &amp; Johnson, Pfizer, Dr Reddy`s)  
+  - Fundaciones y ONGs (Fundación en acción, Fundación ViDa, Asociación Chilena de Agrupaciones Oncológicas, Corporacion Valientes, Tecnigen)  
+  - Empresas de tecnología y diagnóstico (PEGASI DE CHILE SpA, PACIFIC GENOMICS SPA, sk medical, Bradford Hill Spa)  
+  - Representantes individuales (Andrés Arellano, Jorge Martínez Moya, Orieta Matus, Álvaro Ibarra Valencia, Ana María Araya Figueroa, Elizabeth Mendoza, Boris Álvarez)  
+- **Entidades representadas:** Variaron desde compañías multinacionales hasta fundaciones locales, asociaciones de pacientes y consultoras especializadas en salud oncológica.  
+Este listado refleja la amplia gama de actores interesados en influir en las políticas nacionales de cáncer durante el período documentado, con un enfoque particular en acceso a tratamientos, innovación terapéutica y gestión de recursos en el sistema de salud público chileno. Cada participante aportó perspectivas específicas según su afiliación y los intereses que representaban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:44:55</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">what happens on meet in On May 19, 2026 at 10:00 AM, Alejandro Berkovits
+</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está lo que ocurrió en la reunión del **19 de mayo de 2026 a las 10:00 AM** con Alejandro Berkovits:
+- **Participantes**:  
+  - Alejandro Berkovits (Jefe Agencia Nacional del Cáncer, SSP)  
+  - Ana María Araya Figueroa (Gestor de intereses, representando a sí misma)  
+- **Propósito de la reunión**:  
+  Ana María Araya Figueroa contactó al Ministerio para expresar sus preocupaciones específicas sobre el acceso al tratamiento para pacientes con **cáncer de mama triple negativo**, detallando los siguientes puntos:  
+  1. **Retrasos en la entrega de pembrolizumab**:  
+     - Aunque el medicamento pembrolizumab se entrega desde la resolución que actualizó la RE DAC en octubre de 2025, **no siempre llega a tiempo**, lo que retrasa el tratamiento de las pacientes.  
+     - Señaló que, aunque la distribución se ha centralizado y ahora demora menos que antes, persisten problemas de puntualidad en la entrega.  
+  2. **Falta de recursos y errores en hospitales específicos**:  
+     - Expresó preocupación por la **gestión y falta de recursos** en los hospitales de **La Serena, Sótero del Río y Van Buren**.  
+     - Denunció que el **Hospital de Chillán** está excluyendo indebidamente del tratamiento con pembrolizumab a pacientes que, según el resultado de su biopsia, **sí deberían recibirlo**, indicándoles en su lugar **tamoxifeno** (un tratamiento inadecuado para cáncer de mama triple negativo).  
+  3. **Planos de acción personal**:  
+     - Mencionó que planeaba presentarse ante la **Comisión de Mujeres y Equidad de Género** y la **Comisión de Salud** (coordinada por dos parlamentarios), y que le habría gustado informar personalmente al Dr. Berkovits sobre estos asuntos.  
+  4. **Consultas adicionales planteadas**:  
+     - Sobre **asesoramiento genético** relacionado con el cáncer de mama.  
+     - Sobre la **posible actualización de las canastas GES** para el cáncer de mama.  
+     - Sobre si el **recorte presupuestario en salud** afectaría el financiamiento de drogas o la atención de los pacientes oncológicos.  
+- **Respuesta del Ministerio (según se le comunicó a Ana María)**:  
+  - Se le informó que, **oficialmente**, ningún recorte presupuestario afectará **directamente la atención de las personas**.  
+  - Sin embargo, se le sugirió **reiterar todas sus consultas** (incluyendo las mencionadas anteriormente) a través del mecanismo de **Transparencia**, donde recibiría una respuesta más detallada en un plazo de algunos días.  
+- **Detalles técnicos de la reunión**:  
+  - **Identificador**: AO001AW2179080  
+  - **Plataforma**: Videoconferencia mediante Zoom (Enlace: https://minsal-cl.zoom.us/j/85649906536, Contraseña: 323352)  
+  - **Duración**: 1 hora, 0 minutos  
+  - **Tema discutido**: Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos.  
+  - **Fuente**: https://www.leylobby.gob.cl/instituciones/AO001/audiencias/2026/903081/911908  
+En resumen, la reunión se centró en las barreras de acceso al tratamiento oncológico específico para cáncer de mama triple negativo, con énfasis en fallas operativas en la distribución de medicamentos y inequidades territoriales en la atención, concluyendo con una orientación para canalizar las inquietudes mediante vías oficiales de transparencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-08 16:48:08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">what happens on meet in On May 19, 2026 at 10:00 AM, Alejandro Berkovits
+</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está lo que ocurrió en la reunión del **19 de mayo de 2026 a las 10:00 AM** con Alejandro Berkovits (Jefe Agencia Nacional del Cáncer, SSP):
+- **Participante principal**: Ana María Araya Figueroa (representando a sí misma como gestora de intereses) asistió a la videoconferencia para expresar sus preocupaciones relacionadas con el cáncer de mama triple negativo.
+- **Temas centrales discutidos**:
+  - **Retrasos en la entrega de pembrolizumab**: Ana María explicó que, aunque el medicamento pembrolizumab está disponible desde la resolución que actualizó la RE DAC en octubre de 2025, su distribución no siempre llega a tiempo, lo que retrata el tratamiento de las pacientes. Señaló que, aunque la distribución se ha centralizado y ahora es más rápida que antes, persisten demoras críticas.
+  - **Problemas de gestión y recursos hospitalarios**: Expresó preocupación por la falta de recursos y la gestión inadecuada en los hospitales de La Serena, Sótero del Río y Van Buren. Destacó específicamente que el Hospital de Chillán está excluyendo de tratamiento con pembrolizumab a pacientes que, según el resultado de su biopsia, deberían recibirlo, indicándoles en su lugar tamoxifeno.
+  - **Planos personales de advocacy**: Mencionó que planeaba presentarse ante la Comisión de Mujeres y Equidad de Género y la Comisión de Salud (coordinada por dos parlamentarios), y que habría preferido informar personalmente al Dr. Berkovits sobre estos asuntos.
+  - **Consultas adicionales planteadas**:
+    - Temas de asesoramiento genético.
+    - Posible actualización de las canastas GES para el cáncer de mama.
+    - Impacto del recorte presupuestario en salud sobre el financiamiento de drogas o la atención de pacientes oncológicos.
+- **Respuesta del Ministerio**: Se le informó a Ana María que, según la información oficial del Ministerio, ningún recorte presupuestario afectará directamente la atención de las personas. Sin embargo, se le sugirió reiterar todas sus consultas (incluyendo las mencionadas anteriormente) a través del mecanismo de Transparencia, para obtener respuestas más detalladas en un plazo de algunos días.
+- **Detalles técnicos de la reunión**:
+  - **Identificador de la reunión**: AO001AW2179080
+  - **Plataforma**: Videoconferencia mediante Zoom (enlace: https://minsal-cl.zoom.us/j/85649906536, contraseña: 323352), con nota de que no fue posible realizarla de manera presencial debido a dificultades en la agenda.
+  - **Duración**: 1 hora y 0 minutos.
+  - **Asunto tratado**: Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos.
+  - **Enlace de fuente**: https://www.leylobby.gob.cl/instituciones/AO001/audiencias/2026/903081/911908
+Esta reunión se centró en desafíos específicos de acceso al tratamiento para el cáncer de mama triple negativo, con énfasis en barreras logísticas, inequidades territoriales y preocupaciones sobre la adherencia a protocolos clínicos establecidos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:19:13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>what happens on meet in On May 19, 2026 at 10:00 AM, Alejandro Berkovits</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado, aquí está el detalle de lo que ocurrió en la reunión del **19 de mayo de 2026 a las 10:00 AM** con Alejandro Berkovits:
+**Detalles de la reunión:**
+- **Fecha y hora:** 19 de mayo de 2026 a las 10:00 AM
+- **Participante principal:** Ana María Araya Figueroa (representando a sí misma como gestora de intereses)
+- **Plataforma:** Videoconferencia mediante Zoom (Enlace: https://minsal-cl.zoom.us/j/85649906536, Contraseña: 323352)
+- **Duración:** 1 hora
+- **Tema central:** Diseño, implementación y evaluación de políticas, planes y programas efectuados por los sujetos pasivos
+**Lo que sucedió en la reunión (según el propósito documentado):**
+1. **Preocupación por acceso oportuno a pembrolizumab en cáncer de mama triple negativo:**
+   - Ana María explicó que, aunque el medicamento pembrolizumab está disponible desde la resolución que actualizó la RE DAC en octubre de 2025, su entrega no siempre es oportuna, lo que retrasa el tratamiento de las pacientes.
+   - Señaló que, pese a los retrasos, la distribución se ha centralizado y actualmente demora menos que antes.
+2. **Problemas de gestión y recursos en hospitales específicos:**
+   - Expresó preocupación por la gestión y falta de recursos en los hospitales de La Serena, Sótero del Río y Van Buren.
+   - Destacó una situación crítica en el Hospital de Chillán: están excluyendo del tratamiento con pembrolizumab a pacientes que, según el resultado de su biopsia, deberían recibirlo, indicándoles en su lugar tamoxifeno (un tratamiento diferente y menos adecuado para este subtipo de cáncer).
+3. **Planos de participación en instancias gubernamentales:**
+   - Ana María mencionó que se presentaría ante la Comisión de Mujeres y Equidad de Género y ante la Comisión de Salud (coordinada por dos parlamentarios), expresando su deseo de haber podido informar personalmente al Dr. Berkovits sobre estos temas.
+4. **Consultas adicionales planteadas:**
+   - Asesoramiento genético para pacientes oncológicas.
+   - Posible actualización de las canastas GES (Garantías Explícitas en Salud) específicamente para el cáncer de mama.
+   - Impacto del recorte presupuestario en salud sobre el financiamiento de drogas y la atención a pacientes oncológicos.
+5. **Respuesta del Ministerio de Salud (por intermedio de los presentes):**
+   - Se le informó a Ana María que, según la información oficial del Ministerio, ningún recorte presupuestario afectará directamente la atención de las personas.
+   - Sin embargo, se le sugirió reiterar todas sus consultas (incluyendo las mencionadas anteriormente) a través del mecanismo de Transparencia, para obtener respuestas más detalladas en un plazo de algunos días.
+**Identificadores clave de la reunión:**
+- **Identificador de reunión:** AO001AW2179080
+- **Enlace de fuente:** https://www.leylobby.gob.cl/instituciones/AO001/audiencias/2026/903081/911908
+Esta reunión se centró específicamente en los desafíos de acceso a tratamientos oncológicos específicos (pembrolizumab para cáncer de mama triple negativo) y en problemas operativos en hospitales regionales, reflejando preocupaciones concretas de pacientes y defensores sobre la implementación de políticas nacionales de cáncer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-08 17:20:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>who are the participants in this above meetings</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Basado en el contexto proporcionado específicamente para la reunión del **19 de mayo de 2026 a las 10:00 AM** con Alejandro Berkovits, los participantes fueron:
+- **Ana María Araya Figueroa**  
+  (Gestor de intereses, trabajando de forma independiente - "working for nan", representando a sí misma como gestora de intereses)
+**Detalles adicionales sobre la participación:**
+- Ella asistió a la reunión en representación de sus propias preocupaciones como defensora de pacientes oncológicas, específicamente enfocada en el acceso al pembrolizumab para cáncer de mama triple negativo.
+- No se mencionaron otros participantes oficiales del Ministerio de Salud (como Alejandro Berkovits) en la lista de "participantes" del contexto, aunque el contexto indica que él asistió como "Jefe Agencia Nacional del Cáncer, SSP".
+- La reunión se realizó mediante videoconferencia en Zoom, con el enlace y contraseña proporcionados en el contexto.
+**Nota importante:** Aunque el contexto menciona que Alejandro Berkovits asistió a la reunión, la sección específica de "Participantes" en el documento solo lista a Ana María Araya Figueroa. Esto es común en los registros de audiencias de lobby, donde se detallan principalmente los representantes externos que solicitaron la reunión, mientras que los funcionarios gubernamentales presentes se implícitan por el contexto de la reunión (en este caso, Alejandro Berkovits como funcionario del Ministerio de Salud que atendió la solicitud).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>